<commit_message>
Initial commit - timetable system
</commit_message>
<xml_diff>
--- a/ENGLISH_timetable.xlsx
+++ b/ENGLISH_timetable.xlsx
@@ -613,7 +613,11 @@
           <t>6E ENGLISH</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>10B ENGLISH</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
           <t>8B ENGLISH</t>
@@ -691,14 +695,10 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>8C ENGLISH</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>10B ENGLISH</t>
-        </is>
-      </c>
+          <t>6B ENGLISH</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
           <t>7A ENGLISH</t>
@@ -747,17 +747,17 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>8C ENGLISH</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>6D S.ST</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>7D ENGLISH</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>6D S.ST</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>6B ENGLISH</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>6B ENGLISH</t>
+          <t>7D ENGLISH</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr"/>
@@ -916,11 +916,7 @@
           <t>10:10-10:50</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>7D ENGLISH</t>
-        </is>
-      </c>
+      <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -966,17 +962,17 @@
           <t>11:20-12:00</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr"/>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>8C ENGLISH</t>
+        </is>
+      </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
           <t>6C ENGLISH</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>8C ENGLISH</t>
-        </is>
-      </c>
+      <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1042,7 +1038,11 @@
           <t>6D ENGLISH</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>6B ENGLISH</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
           <t>9A ENGLISH</t>
@@ -1263,11 +1263,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>8C ENGLISH</t>
-        </is>
-      </c>
+      <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
           <t>9A ENGLISH</t>
@@ -1364,11 +1360,15 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
+          <t>8C ENGLISH</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
           <t>7D ENGLISH</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
           <t>10E ENGLISH</t>
@@ -1498,17 +1498,17 @@
           <t>10:40-11:15</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>8C ENGLISH</t>
+        </is>
+      </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
           <t>7B ENGLISH</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>8C ENGLISH</t>
-        </is>
-      </c>
+      <c r="F37" s="2" t="inlineStr"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
           <t>9A ENGLISH</t>
@@ -1601,7 +1601,11 @@
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>7D ENGLISH</t>
+        </is>
+      </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
           <t>10E ENGLISH</t>
@@ -1653,11 +1657,7 @@
           <t>1:15-2:00</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>7D ENGLISH</t>
-        </is>
-      </c>
+      <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr">
         <is>
           <t>6D ENGLISH</t>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>7D ENGLISH</t>
+          <t>8C ENGLISH</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -1861,7 +1861,11 @@
           <t>8A ENGLISH</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>7D ENGLISH</t>
+        </is>
+      </c>
       <c r="G48" s="2" t="inlineStr"/>
       <c r="H48" s="2" t="inlineStr"/>
       <c r="I48" s="2" t="inlineStr">
@@ -1888,11 +1892,7 @@
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr"/>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>8C ENGLISH</t>
-        </is>
-      </c>
+      <c r="F49" s="2" t="inlineStr"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
           <t>9D ENGLISH</t>

</xml_diff>